<commit_message>
proper label creation using json
</commit_message>
<xml_diff>
--- a/schema.xlsx
+++ b/schema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Findlay\Desktop\My stuff\Coding\Rust\inventorize\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97DECCDA-8180-45F4-9DB9-FF381CA0B24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D464C9-252C-4BDD-B6EC-2AB7296CB522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1185" windowWidth="28800" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Components</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>prompts</t>
+  </si>
+  <si>
+    <t>{resistance: [R], size: [S], value: [V], materials: {casing: "Metal", conductor: "Thick Film"}}</t>
   </si>
 </sst>
 </file>
@@ -99,8 +102,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,7 +391,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.5703125" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="35.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:12" x14ac:dyDescent="0.25">
@@ -425,6 +432,11 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:12" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="6" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
typing (desperately) to add json support
</commit_message>
<xml_diff>
--- a/schema.xlsx
+++ b/schema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Findlay\Desktop\My stuff\Coding\Rust\inventorize\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D464C9-252C-4BDD-B6EC-2AB7296CB522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{173C106E-92B3-4971-B0D1-4AC9DA7A9279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1185" windowWidth="28800" windowHeight="11115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Components</t>
   </si>
@@ -67,6 +67,21 @@
   </si>
   <si>
     <t>{resistance: [R], size: [S], value: [V], materials: {casing: "Metal", conductor: "Thick Film"}}</t>
+  </si>
+  <si>
+    <t>{attributes: [{name: "resistance", unit: "ohm"}, {name: "capacitance", unit: "F"}]}</t>
+  </si>
+  <si>
+    <t>{prompts: {resistance: [{value: 60, count: 8},{value: 80, count: 5}]}}</t>
+  </si>
+  <si>
+    <t>schema</t>
+  </si>
+  <si>
+    <t>{type: "object", properties: {resistance: {type: "integer"}, package: {type: "string"}}}</t>
+  </si>
+  <si>
+    <t>resistor</t>
   </si>
 </sst>
 </file>
@@ -102,10 +117,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -387,10 +408,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:L7"/>
+  <dimension ref="C3:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" customWidth="1"/>
     <col min="11" max="11" width="13.5703125" customWidth="1"/>
     <col min="12" max="12" width="35.5703125" customWidth="1"/>
   </cols>
@@ -433,6 +457,9 @@
       </c>
     </row>
     <row r="5" spans="3:12" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K5" s="3">
+        <v>0</v>
+      </c>
       <c r="L5" s="1" t="s">
         <v>13</v>
       </c>
@@ -442,7 +469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>1</v>
       </c>
@@ -453,7 +480,27 @@
         <v>7</v>
       </c>
       <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="3:12" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>